<commit_message>
Play-test 14 (lane D): ten bosses deleted, their story slots taken by kept bosses
Hive->Matriarch, Atlas->Behemoth Mk.II, Kronos->Tartarus, Caspian->Charybdis, Morrigan->Harpy, Spectre->Roc,
Gungnir->Monster; data, campaign, strings, tests, xlsx; models archived (Docs/fixes/playtest14_deleted.md).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/balance/Machine_Brigade_Can_bang_dot2_v2.xlsx
+++ b/Docs/balance/Machine_Brigade_Can_bang_dot2_v2.xlsx
@@ -22842,55 +22842,24 @@
       </c>
     </row>
     <row r="360" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A360" s="13" t="s">
-        <v>926</v>
-      </c>
-      <c r="B360" s="13" t="s">
-        <v>927</v>
-      </c>
-      <c r="C360" s="13" t="s">
-        <v>928</v>
-      </c>
-      <c r="D360" s="13" t="s">
-        <v>929</v>
-      </c>
-      <c r="E360" s="13" t="s">
-        <v>128</v>
-      </c>
+      <c r="A360" s="13"/>
+      <c r="B360" s="13"/>
+      <c r="C360" s="13"/>
+      <c r="D360" s="13"/>
+      <c r="E360" s="13"/>
       <c r="F360" s="13"/>
-      <c r="G360" s="13" t="n">
-        <v>400</v>
-      </c>
-      <c r="H360" s="13" t="n">
-        <v>180</v>
-      </c>
+      <c r="G360" s="13"/>
+      <c r="H360" s="13"/>
       <c r="I360" s="13"/>
-      <c r="J360" s="13" t="s">
-        <v>930</v>
-      </c>
-      <c r="K360" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="L360" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="M360" s="16" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
+      <c r="J360" s="13"/>
+      <c r="K360" s="19"/>
+      <c r="L360" s="13"/>
+      <c r="M360" s="16"/>
       <c r="N360" s="13"/>
-      <c r="O360" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="P360" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q360" s="13" t="s">
-        <v>930</v>
-      </c>
-      <c r="R360" s="13" t="s">
-        <v>931</v>
-      </c>
+      <c r="O360" s="13"/>
+      <c r="P360" s="13"/>
+      <c r="Q360" s="13"/>
+      <c r="R360" s="13"/>
     </row>
     <row r="361" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="13"/>
@@ -25640,21 +25609,11 @@
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="13" t="s">
-        <v>926</v>
-      </c>
-      <c r="B152" s="13" t="s">
-        <v>927</v>
-      </c>
-      <c r="C152" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D152" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="E152" s="13" t="s">
-        <v>960</v>
-      </c>
+      <c r="A152" s="13"/>
+      <c r="B152" s="13"/>
+      <c r="C152" s="13"/>
+      <c r="D152" s="19"/>
+      <c r="E152" s="13"/>
       <c r="F152" s="13"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>